<commit_message>
Auto update RUP 23/06/2026 11:00:30,85
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-23) Legacy.xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-23) Legacy.xlsx
@@ -2129,19 +2129,19 @@
         <v>887410440</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>892410440</v>
+        <v>887410440</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>892410440</v>
+        <v>887410440</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>100.5634371396397</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61">

</xml_diff>